<commit_message>
도 감 구 현 성 공 !!!!!!!!!!!!!!!
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Item.xlsx
+++ b/JsonConverter/ExcelFiles/Item.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t xml:space="preserve">캐릭터 고유 ID</t>
   </si>
@@ -52,6 +52,9 @@
     <t xml:space="preserve">PrefabPath</t>
   </si>
   <si>
+    <t xml:space="preserve">CollectionId</t>
+  </si>
+  <si>
     <t xml:space="preserve">obj_cherry_01</t>
   </si>
   <si>
@@ -77,6 +80,9 @@
   </si>
   <si>
     <t xml:space="preserve">Collective/obj_collecton_gem_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collection_gem_01</t>
   </si>
 </sst>
 </file>
@@ -223,6 +229,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -249,10 +259,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -527,77 +533,81 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.78"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="15" min="7" style="1" width="12.65"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16381" min="18" style="1" width="12.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16382" min="16382" style="0" width="11.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16382" min="16382" style="3" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="5" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" s="9" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="F2" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" s="10" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="XFB3" s="0"/>
+      <c r="F3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="XFB3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="D4" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="E4" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F4" s="4"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
@@ -610,19 +620,21 @@
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>17</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="12"/>
+        <v>19</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="G5" s="12"/>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
@@ -634,10 +646,10 @@
       <c r="O5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="4"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -651,10 +663,10 @@
       <c r="O6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="4"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -668,10 +680,10 @@
       <c r="O7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="4"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -685,10 +697,10 @@
       <c r="O8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -702,10 +714,10 @@
       <c r="O9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="4"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -719,10 +731,10 @@
       <c r="O10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="4"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -736,10 +748,10 @@
       <c r="O11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="4"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="5"/>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -753,10 +765,10 @@
       <c r="O12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="5"/>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
@@ -770,10 +782,10 @@
       <c r="O13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="4"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="5"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>

</xml_diff>